<commit_message>
Prazo FNE de 14 anos pela condição de administração majoritariamente feminina
Recalcula viabilidade e capacidade de pagamento com 14 anos/4 carência
(FNE Mulher): pleito integral passa na janela do BNB com preço R$ 82/t
(47,0%); máximo financiável na receita-base sobe a R$ 21,9 mi. Projeção
estendida a 14 anos (TIR 14,9%, VPL R$ 4,9 mi, DSCR mín 1,29). Atualiza
XLSX, relatório de viabilidade, plano de produção e verificação de
licenças; documenta exigência de comprovação societária da condição.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DqEaERD1LDFtugtNrL73cp
</commit_message>
<xml_diff>
--- a/Viabilidade_CIPREM.xlsx
+++ b/Viabilidade_CIPREM.xlsx
@@ -606,14 +606,14 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2) CAPACIDADE: com receita-base e 12 anos, o pleito integral de R$ 24,29 mi NÃO passa na janela de 50% (comprometimento 63,9%).</t>
+          <t>2) CAPACIDADE: prazo de 14 anos garantido pela condição FNE Mulher (adm. majoritariamente feminina). Com receita-base,</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Caminhos que passam: 15 anos/4 carência + preço médio R$ 82/t (42,7%) OU reduzir pleito a ~R$ 20 mi em 12 anos.</t>
+          <t xml:space="preserve">   o pleito integral compromete 57,3% (não passa); com preço médio R$ 82/t passa com 47,0%. Alternativa: pleito ~R$ 21,9 mi.</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>BASE (preço 68,50 · 12a/3c)</t>
+          <t>BASE (preço 68,50 · 14a/4c)</t>
         </is>
       </c>
       <c r="B4" s="14" t="n">
@@ -740,14 +740,14 @@
         <v>0.3628904223838094</v>
       </c>
       <c r="F4" s="15" t="n">
-        <v>0.1357531417410779</v>
+        <v>0.1494322271217648</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>2345299.887343785</v>
+        <v>4927889.77581582</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>63,9% ✗</t>
+          <t>57,3% ✗</t>
         </is>
       </c>
     </row>
@@ -770,10 +770,10 @@
         <v>-0.1933564539104353</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>0.06083644203130134</v>
+        <v>0.07908943923859313</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-8078531.973660741</v>
+        <v>-6303892.299403776</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
@@ -800,10 +800,10 @@
         <v>-0.1862707733603469</v>
       </c>
       <c r="F6" s="15" t="n">
-        <v>0.05458978611840293</v>
+        <v>0.07325198415876433</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-8837722.548969323</v>
+        <v>-7129164.450326623</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
@@ -827,13 +827,13 @@
         <v>-2574535.5212</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>0.3606093833557695</v>
+        <v>0.3628904223838094</v>
       </c>
       <c r="F7" s="15" t="n">
-        <v>-0.03311555848232023</v>
+        <v>-0.009372448266384226</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-15540268.75834021</v>
+        <v>-14776093.99485386</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
@@ -860,21 +860,21 @@
         <v>0.6893739127119133</v>
       </c>
       <c r="F8" s="15" t="n">
-        <v>0.2093424394212383</v>
+        <v>0.2194947337644882</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>14671595.34553619</v>
+        <v>18315725.66144409</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>42,7% ✓ (15a/4c)</t>
+          <t>47,0% ✓ (14a/4c)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Recomendação: estruturar o pleito em 15 anos/4 carência e defender preço médio ≥ R$ 82/t (PVV realiza R$ 116/t bruto blended), OU reduzir o pleito a ~R$ 20 mi em 12 anos.</t>
+          <t>Recomendação: pleito em 14 anos/4 carência (direito pela condição FNE Mulher) + defender preço médio ≥ R$ 82/t (PVV realiza R$ 116/t bruto), OU reduzir o pleito a ~R$ 21,9 mi.</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:P39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -907,6 +907,8 @@
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1152,6 +1154,12 @@
       <c r="N21" s="6" t="n">
         <v>19</v>
       </c>
+      <c r="O21" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="P21" s="6" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1195,6 +1203,12 @@
       <c r="N22" s="10" t="n">
         <v>1100000</v>
       </c>
+      <c r="O22" s="10" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="P22" s="10" t="n">
+        <v>1100000</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1238,6 +1252,12 @@
       <c r="N23" s="10" t="n">
         <v>1500000</v>
       </c>
+      <c r="O23" s="10" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="P23" s="10" t="n">
+        <v>1500000</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1308,11 +1328,11 @@
         </is>
       </c>
       <c r="B31" s="12" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>testar 15 na Capacidade_BNB</t>
+          <t>14 anos — condição FNE Mulher (adm. majoritariamente feminina); comprovar no contrato social</t>
         </is>
       </c>
     </row>
@@ -1323,7 +1343,7 @@
         </is>
       </c>
       <c r="B32" s="12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33">
@@ -1419,6 +1439,16 @@
           <t>Ano 12</t>
         </is>
       </c>
+      <c r="O37" s="13" t="inlineStr">
+        <is>
+          <t>Ano 13</t>
+        </is>
+      </c>
+      <c r="P37" s="13" t="inlineStr">
+        <is>
+          <t>Ano 14</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -1460,6 +1490,12 @@
         <v>216000</v>
       </c>
       <c r="N38" s="8" t="n">
+        <v>216000</v>
+      </c>
+      <c r="O38" s="8" t="n">
+        <v>216000</v>
+      </c>
+      <c r="P38" s="8" t="n">
         <v>216000</v>
       </c>
     </row>
@@ -1822,7 +1858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1839,6 +1875,8 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1909,6 +1947,16 @@
           <t>Ano 12</t>
         </is>
       </c>
+      <c r="O3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 13</t>
+        </is>
+      </c>
+      <c r="P3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 14</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1964,6 +2012,14 @@
         <f>Premissas!N$38</f>
         <v/>
       </c>
+      <c r="O4" s="18">
+        <f>Premissas!O$38</f>
+        <v/>
+      </c>
+      <c r="P4" s="18">
+        <f>Premissas!P$38</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2019,6 +2075,14 @@
         <f>MIN(N4*Premissas!$B$13,Premissas!$B$14)</f>
         <v/>
       </c>
+      <c r="O5" s="18">
+        <f>MIN(O4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="P5" s="18">
+        <f>MIN(P4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2074,6 +2138,14 @@
         <f>N4*Premissas!$B$10</f>
         <v/>
       </c>
+      <c r="O6" s="19">
+        <f>O4*Premissas!$B$10</f>
+        <v/>
+      </c>
+      <c r="P6" s="19">
+        <f>P4*Premissas!$B$10</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -2129,6 +2201,14 @@
         <f>N5*Premissas!$B$15</f>
         <v/>
       </c>
+      <c r="O7" s="19">
+        <f>O5*Premissas!$B$15</f>
+        <v/>
+      </c>
+      <c r="P7" s="19">
+        <f>P5*Premissas!$B$15</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -2184,6 +2264,14 @@
         <f>N6+N7</f>
         <v/>
       </c>
+      <c r="O8" s="14">
+        <f>O6+O7</f>
+        <v/>
+      </c>
+      <c r="P8" s="14">
+        <f>P6+P7</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -2239,6 +2327,14 @@
         <f>-N8*Premissas!$B$17</f>
         <v/>
       </c>
+      <c r="O9" s="19">
+        <f>-O8*Premissas!$B$17</f>
+        <v/>
+      </c>
+      <c r="P9" s="19">
+        <f>-P8*Premissas!$B$17</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -2292,6 +2388,14 @@
       </c>
       <c r="N10" s="14">
         <f>N8+N9</f>
+        <v/>
+      </c>
+      <c r="O10" s="14">
+        <f>O8+O9</f>
+        <v/>
+      </c>
+      <c r="P10" s="14">
+        <f>P8+P9</f>
         <v/>
       </c>
     </row>
@@ -2306,7 +2410,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2323,6 +2427,8 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2393,6 +2499,16 @@
           <t>Ano 12</t>
         </is>
       </c>
+      <c r="O3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 13</t>
+        </is>
+      </c>
+      <c r="P3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 14</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -2448,6 +2564,14 @@
         <f>Producao_Receita!N4*Premissas!N$21</f>
         <v/>
       </c>
+      <c r="O4" s="19">
+        <f>Producao_Receita!O4*Premissas!O$21</f>
+        <v/>
+      </c>
+      <c r="P4" s="19">
+        <f>Producao_Receita!P4*Premissas!P$21</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2503,6 +2627,14 @@
         <f>Producao_Receita!N7*Premissas!$B$16</f>
         <v/>
       </c>
+      <c r="O5" s="19">
+        <f>Producao_Receita!O7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="P5" s="19">
+        <f>Producao_Receita!P7*Premissas!$B$16</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -2558,6 +2690,14 @@
         <f>Producao_Receita!N8*Premissas!$B$18</f>
         <v/>
       </c>
+      <c r="O6" s="19">
+        <f>Producao_Receita!O8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="P6" s="19">
+        <f>Producao_Receita!P8*Premissas!$B$18</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -2613,6 +2753,14 @@
         <f>Premissas!N$22</f>
         <v/>
       </c>
+      <c r="O7" s="19">
+        <f>Premissas!O$22</f>
+        <v/>
+      </c>
+      <c r="P7" s="19">
+        <f>Premissas!P$22</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2668,6 +2816,14 @@
         <f>Premissas!N$23</f>
         <v/>
       </c>
+      <c r="O8" s="19">
+        <f>Premissas!O$23</f>
+        <v/>
+      </c>
+      <c r="P8" s="19">
+        <f>Premissas!P$23</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -2723,6 +2879,14 @@
         <f>Premissas!$B$24</f>
         <v/>
       </c>
+      <c r="O9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="P9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -2776,6 +2940,14 @@
       </c>
       <c r="N10" s="19">
         <f>SUM(N4:N9)</f>
+        <v/>
+      </c>
+      <c r="O10" s="19">
+        <f>SUM(O4:O9)</f>
+        <v/>
+      </c>
+      <c r="P10" s="19">
+        <f>SUM(P4:P9)</f>
         <v/>
       </c>
     </row>
@@ -2790,7 +2962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2807,6 +2979,8 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2877,6 +3051,16 @@
           <t>Ano 12</t>
         </is>
       </c>
+      <c r="O3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 13</t>
+        </is>
+      </c>
+      <c r="P3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 14</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -2932,6 +3116,14 @@
         <f>M7</f>
         <v/>
       </c>
+      <c r="O4" s="14">
+        <f>N7</f>
+        <v/>
+      </c>
+      <c r="P4" s="14">
+        <f>O7</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2987,6 +3179,14 @@
         <f>N4*Premissas!$B$33</f>
         <v/>
       </c>
+      <c r="O5" s="14">
+        <f>O4*Premissas!$B$33</f>
+        <v/>
+      </c>
+      <c r="P5" s="14">
+        <f>P4*Premissas!$B$33</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -3042,6 +3242,14 @@
         <f>IF(12&gt;Premissas!$B$32,Premissas!$B$30/(Premissas!$B$31-Premissas!$B$32),0)</f>
         <v/>
       </c>
+      <c r="O6" s="14">
+        <f>IF(13&gt;Premissas!$B$32,Premissas!$B$30/(Premissas!$B$31-Premissas!$B$32),0)</f>
+        <v/>
+      </c>
+      <c r="P6" s="14">
+        <f>IF(14&gt;Premissas!$B$32,Premissas!$B$30/(Premissas!$B$31-Premissas!$B$32),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -3097,6 +3305,14 @@
         <f>N4-N6</f>
         <v/>
       </c>
+      <c r="O7" s="14">
+        <f>O4-O6</f>
+        <v/>
+      </c>
+      <c r="P7" s="14">
+        <f>P4-P6</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -3150,6 +3366,14 @@
       </c>
       <c r="N8" s="14">
         <f>N5+N6</f>
+        <v/>
+      </c>
+      <c r="O8" s="14">
+        <f>O5+O6</f>
+        <v/>
+      </c>
+      <c r="P8" s="14">
+        <f>P5+P6</f>
         <v/>
       </c>
     </row>
@@ -3164,7 +3388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3181,6 +3405,8 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3251,6 +3477,16 @@
           <t>Ano 12</t>
         </is>
       </c>
+      <c r="O3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 13</t>
+        </is>
+      </c>
+      <c r="P3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 14</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -3306,6 +3542,14 @@
         <f>Producao_Receita!N8</f>
         <v/>
       </c>
+      <c r="O4" s="19">
+        <f>Producao_Receita!O8</f>
+        <v/>
+      </c>
+      <c r="P4" s="19">
+        <f>Producao_Receita!P8</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -3361,6 +3605,14 @@
         <f>Producao_Receita!N9</f>
         <v/>
       </c>
+      <c r="O5" s="19">
+        <f>Producao_Receita!O9</f>
+        <v/>
+      </c>
+      <c r="P5" s="19">
+        <f>Producao_Receita!P9</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -3416,6 +3668,14 @@
         <f>Producao_Receita!N10</f>
         <v/>
       </c>
+      <c r="O6" s="19">
+        <f>Producao_Receita!O10</f>
+        <v/>
+      </c>
+      <c r="P6" s="19">
+        <f>Producao_Receita!P10</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -3471,6 +3731,14 @@
         <f>-Custos!N10</f>
         <v/>
       </c>
+      <c r="O7" s="19">
+        <f>-Custos!O10</f>
+        <v/>
+      </c>
+      <c r="P7" s="19">
+        <f>-Custos!P10</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -3526,6 +3794,14 @@
         <f>N6+N7</f>
         <v/>
       </c>
+      <c r="O8" s="19">
+        <f>O6+O7</f>
+        <v/>
+      </c>
+      <c r="P8" s="19">
+        <f>P6+P7</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -3581,6 +3857,14 @@
         <f>IFERROR(N8/N6,0)</f>
         <v/>
       </c>
+      <c r="O9" s="20">
+        <f>IFERROR(O8/O6,0)</f>
+        <v/>
+      </c>
+      <c r="P9" s="20">
+        <f>IFERROR(P8/P6,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -3636,6 +3920,14 @@
         <f>-Premissas!$B$25</f>
         <v/>
       </c>
+      <c r="O10" s="19">
+        <f>-Premissas!$B$25</f>
+        <v/>
+      </c>
+      <c r="P10" s="19">
+        <f>-Premissas!$B$25</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -3691,6 +3983,14 @@
         <f>-FNE_SAC!N5</f>
         <v/>
       </c>
+      <c r="O11" s="19">
+        <f>-FNE_SAC!O5</f>
+        <v/>
+      </c>
+      <c r="P11" s="19">
+        <f>-FNE_SAC!P5</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -3746,6 +4046,14 @@
         <f>N8+N10+N11</f>
         <v/>
       </c>
+      <c r="O12" s="19">
+        <f>O8+O10+O11</f>
+        <v/>
+      </c>
+      <c r="P12" s="19">
+        <f>P8+P10+P11</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -3801,6 +4109,14 @@
         <f>-(0.15*(0.08*N4)+0.1*MAX(0,0.08*N4-240000)+0.09*(0.12*N4))</f>
         <v/>
       </c>
+      <c r="O13" s="19">
+        <f>-(0.15*(0.08*O4)+0.1*MAX(0,0.08*O4-240000)+0.09*(0.12*O4))</f>
+        <v/>
+      </c>
+      <c r="P13" s="19">
+        <f>-(0.15*(0.08*P4)+0.1*MAX(0,0.08*P4-240000)+0.09*(0.12*P4))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -3854,6 +4170,14 @@
       </c>
       <c r="N14" s="19">
         <f>N12+N13</f>
+        <v/>
+      </c>
+      <c r="O14" s="19">
+        <f>O12+O13</f>
+        <v/>
+      </c>
+      <c r="P14" s="19">
+        <f>P12+P13</f>
         <v/>
       </c>
     </row>
@@ -3868,7 +4192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3885,6 +4209,8 @@
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3960,6 +4286,16 @@
           <t>Ano 12</t>
         </is>
       </c>
+      <c r="O3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 13</t>
+        </is>
+      </c>
+      <c r="P3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 14</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -4015,6 +4351,14 @@
         <f>MAX(0,(Producao_Receita!N8-Producao_Receita!M8)*Premissas!$B$26)</f>
         <v/>
       </c>
+      <c r="O4" s="14">
+        <f>MAX(0,(Producao_Receita!O8-Producao_Receita!N8)*Premissas!$B$26)</f>
+        <v/>
+      </c>
+      <c r="P4" s="14">
+        <f>MAX(0,(Producao_Receita!P8-Producao_Receita!O8)*Premissas!$B$26)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -4074,6 +4418,14 @@
         <f>DRE_Projetada!N8+DRE_Projetada!N13-N4</f>
         <v/>
       </c>
+      <c r="O5" s="19">
+        <f>DRE_Projetada!O8+DRE_Projetada!O13-O4</f>
+        <v/>
+      </c>
+      <c r="P5" s="19">
+        <f>DRE_Projetada!P8+DRE_Projetada!P13-P4</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -4133,6 +4485,14 @@
         <f>N5-FNE_SAC!N8</f>
         <v/>
       </c>
+      <c r="O6" s="19">
+        <f>O5-FNE_SAC!O8</f>
+        <v/>
+      </c>
+      <c r="P6" s="19">
+        <f>P5-FNE_SAC!P8</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -4192,6 +4552,14 @@
         <f>M7+N5</f>
         <v/>
       </c>
+      <c r="O7" s="14">
+        <f>N7+O5</f>
+        <v/>
+      </c>
+      <c r="P7" s="14">
+        <f>O7+P5</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -4247,6 +4615,14 @@
         <f>IFERROR((DRE_Projetada!N8+DRE_Projetada!N13)/FNE_SAC!N8,"—")</f>
         <v/>
       </c>
+      <c r="O8" s="17">
+        <f>IFERROR((DRE_Projetada!O8+DRE_Projetada!O13)/FNE_SAC!O8,"—")</f>
+        <v/>
+      </c>
+      <c r="P8" s="17">
+        <f>IFERROR((DRE_Projetada!P8+DRE_Projetada!P13)/FNE_SAC!P8,"—")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -4262,7 +4638,7 @@
         </is>
       </c>
       <c r="B11" s="22">
-        <f>IRR(B5:N5)</f>
+        <f>IRR(B5:P5)</f>
         <v/>
       </c>
     </row>
@@ -4273,7 +4649,7 @@
         </is>
       </c>
       <c r="B12" s="22">
-        <f>IRR(B6:N6)</f>
+        <f>IRR(B6:P6)</f>
         <v/>
       </c>
     </row>
@@ -4284,7 +4660,7 @@
         </is>
       </c>
       <c r="B13" s="23">
-        <f>NPV(Premissas!$B$34,C5:N5)+B5</f>
+        <f>NPV(Premissas!$B$34,C5:P5)+B5</f>
         <v/>
       </c>
     </row>
@@ -4295,7 +4671,7 @@
         </is>
       </c>
       <c r="B14" s="24">
-        <f>COUNTIF(B7:N7,"&lt;0")</f>
+        <f>COUNTIF(B7:P7,"&lt;0")</f>
         <v/>
       </c>
     </row>
@@ -4306,7 +4682,7 @@
         </is>
       </c>
       <c r="B15" s="25">
-        <f>MIN(F8:N8)</f>
+        <f>MIN(G8:P8)</f>
         <v/>
       </c>
     </row>
@@ -4321,7 +4697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -4382,58 +4758,58 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>acima da janela de 50%</t>
+          <t>referência sem a condição Mulher</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Pleito R$ 24,29 mi · 15 anos / 4 carência · receita-base</t>
+          <t>Pleito R$ 24,29 mi · 14 anos / 4 carência · receita-base</t>
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>0.5199774623199154</v>
-      </c>
-      <c r="C6" s="27" t="inlineStr">
-        <is>
-          <t>LIMITE</t>
+        <v>0.5732451073480566</v>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>NÃO PASSA</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>52% — praticamente na janela</t>
+          <t>57,3% — acima da janela</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Pleito R$ 24,29 mi · 15 anos / 4 carência · preço R$ 82/t</t>
+          <t>Pleito R$ 24,29 mi · 14 anos / 3 carência · receita-base</t>
         </is>
       </c>
       <c r="B7" s="15" t="n">
-        <v>0.4267746983765545</v>
-      </c>
-      <c r="C7" s="28" t="inlineStr">
-        <is>
-          <t>PASSA</t>
+        <v>0.5199774623199154</v>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>LIMITE</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>42,7% — dentro da janela</t>
+          <t>52,0% — praticamente na janela</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Pleito R$ 24,29 mi · 15a/4c · preço 82 + teto da licença</t>
+          <t>Pleito R$ 24,29 mi · 14 anos / 4 carência · preço R$ 82/t</t>
         </is>
       </c>
       <c r="B8" s="15" t="n">
-        <v>0.3340595507889639</v>
+        <v>0.4700902764365716</v>
       </c>
       <c r="C8" s="28" t="inlineStr">
         <is>
@@ -4442,49 +4818,69 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>33,4% — folga</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+          <t>47,0% — dentro da janela</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Pleito R$ 24,29 mi · 14a/4c · preço 82 + teto da licença</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>0.3679927983211566</v>
+      </c>
+      <c r="C9" s="28" t="inlineStr">
+        <is>
+          <t>PASSA</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>36,8% — folga</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>FINANCIAMENTO MÁXIMO QUE PASSA (≤50%)</t>
         </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>12 anos / 3 carência · receita-base</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="n">
-        <v>20062332.39690118</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>15 anos / 4 carência · receita-base</t>
+          <t>14 anos / 4 carência · receita-base</t>
         </is>
       </c>
       <c r="B12" s="14" t="n">
-        <v>23573707.46353081</v>
+        <v>21855240.32583817</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>15 anos / 4 carência · preço R$ 82/t</t>
+          <t>14 anos / 4 carência · preço R$ 82/t</t>
         </is>
       </c>
       <c r="B13" s="14" t="n">
-        <v>27512383.80803625</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+        <v>25506796.63585015</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>12 anos / 3 carência · receita-base (referência)</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="n">
+        <v>20062332.39691937</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Formulas sem cache: o Excel recalcula ao abrir. Nota: valores estáticos (o algoritmo do banco não é replicável em fórmula de planilha). Para recalcular após mudar premissas, rodar o script capacidade_pagamento.py da skill do consultor.</t>
         </is>

</xml_diff>

<commit_message>
Montagem 14 anos = 2 carência + 12 amortização: pleito passa na receita-base
Comparativo das montagens no motor oficial BNB: 2c+12a compromete 48,5%
(passa no conservador; 39,8% com preço 82; máx. financiável R$ 24,8 mi >
pleito), vs 52,0% (3c+11a) e 57,3% (4c+10a). Atualiza XLSX (carência 2,
tabela Capacidade_BNB, DSCR range) e relatório (§3 com SAC 2c, §5
comparativo e recomendação com nota de amortização equalizada para o
DSCR 1,13 do ano 3).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DqEaERD1LDFtugtNrL73cp
</commit_message>
<xml_diff>
--- a/Viabilidade_CIPREM.xlsx
+++ b/Viabilidade_CIPREM.xlsx
@@ -77,7 +77,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00C00000"/>
+      <color rgb="002E7D46"/>
       <sz val="10"/>
     </font>
     <font>
@@ -89,7 +89,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="002E7D46"/>
+      <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -606,14 +606,14 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2) CAPACIDADE: prazo de 14 anos garantido pela condição FNE Mulher (adm. majoritariamente feminina). Com receita-base,</t>
+          <t>2) CAPACIDADE: prazo de 14 anos (condição FNE Mulher) montado como 2 de carência + 12 de amortização: o pleito integral</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">   o pleito integral compromete 57,3% (não passa); com preço médio R$ 82/t passa com 47,0%. Alternativa: pleito ~R$ 21,9 mi.</t>
+          <t xml:space="preserve">   passa na janela JÁ NA RECEITA-BASE (48,5%); com preço R$ 82/t sobra colchão (39,8%). Máx. financiável: R$ 24,8 mi.</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>BASE (preço 68,50 · 14a/4c)</t>
+          <t>BASE (preço 68,50 · 14a 2c+12a)</t>
         </is>
       </c>
       <c r="B4" s="14" t="n">
@@ -734,10 +734,10 @@
         <v>6467040</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1617350.7508</v>
+        <v>1799529.3349</v>
       </c>
       <c r="E4" s="17" t="n">
-        <v>0.3628904223838094</v>
+        <v>1.132739598198722</v>
       </c>
       <c r="F4" s="15" t="n">
         <v>0.1494322271217648</v>
@@ -747,7 +747,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>57,3% ✗</t>
+          <t>48,5% ✓</t>
         </is>
       </c>
     </row>
@@ -764,10 +764,10 @@
         <v>4536162</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>-245169.7291999997</v>
+        <v>-62991.14509999985</v>
       </c>
       <c r="E5" s="17" t="n">
-        <v>-0.1933564539104353</v>
+        <v>0.7641002725810009</v>
       </c>
       <c r="F5" s="15" t="n">
         <v>0.07908943923859313</v>
@@ -794,10 +794,10 @@
         <v>4383828</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>-640408.5080000001</v>
+        <v>-437987.8589999999</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>-0.1862707733603469</v>
+        <v>0.6930873485594393</v>
       </c>
       <c r="F6" s="15" t="n">
         <v>0.07325198415876433</v>
@@ -824,10 +824,10 @@
         <v>2019324</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>-2574535.5212</v>
+        <v>-2392356.9371</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>0.3628904223838094</v>
+        <v>0.4373219322438476</v>
       </c>
       <c r="F7" s="15" t="n">
         <v>-0.009372448266384226</v>
@@ -854,10 +854,10 @@
         <v>9003960</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>4064457.950800001</v>
+        <v>4246636.5349</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>0.6893739127119133</v>
+        <v>1.617083237696459</v>
       </c>
       <c r="F8" s="15" t="n">
         <v>0.2194947337644882</v>
@@ -867,14 +867,14 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>47,0% ✓ (14a/4c)</t>
+          <t>39,8% ✓</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Recomendação: pleito em 14 anos/4 carência (direito pela condição FNE Mulher) + defender preço médio ≥ R$ 82/t (PVV realiza R$ 116/t bruto), OU reduzir o pleito a ~R$ 21,9 mi.</t>
+          <t>Recomendação: pleito em 14 anos = 2 carência + 12 amortização (condição FNE Mulher) — passa na receita-base (48,5%); defender preço ≥ R$ 82/t como colchão. Atenção ao DSCR 1,13 do ano 3 (SAC constante): negociar amortização equalizada/crescente, que a própria planilha do banco pratica.</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1343,12 @@
         </is>
       </c>
       <c r="B32" s="12" t="n">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>2+12 — montagem que passa na janela já na receita-base</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -4682,7 +4687,7 @@
         </is>
       </c>
       <c r="B15" s="25">
-        <f>MIN(G8:P8)</f>
+        <f>MIN(E8:P8)</f>
         <v/>
       </c>
     </row>
@@ -4745,47 +4750,47 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Pleito R$ 24,29 mi · 12 anos / 3 carência · receita-base</t>
+          <t>Pleito R$ 24,29 mi · 14a · 2 car + 12 amort · receita-base</t>
         </is>
       </c>
       <c r="B5" s="15" t="n">
-        <v>0.6386693237419049</v>
+        <v>0.4853622760434536</v>
       </c>
       <c r="C5" s="26" t="inlineStr">
         <is>
-          <t>NÃO PASSA</t>
+          <t>PASSA</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>referência sem a condição Mulher</t>
+          <t>48,5% — dentro da janela já no conservador</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Pleito R$ 24,29 mi · 14 anos / 4 carência · receita-base</t>
+          <t>Pleito R$ 24,29 mi · 14a · 2 car + 12 amort · preço R$ 82/t</t>
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>0.5732451073480566</v>
+        <v>0.3977969351818025</v>
       </c>
       <c r="C6" s="26" t="inlineStr">
         <is>
-          <t>NÃO PASSA</t>
+          <t>PASSA</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>57,3% — acima da janela</t>
+          <t>39,8% — colchão</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Pleito R$ 24,29 mi · 14 anos / 3 carência · receita-base</t>
+          <t>Pleito R$ 24,29 mi · 14a · 3 car + 11 amort · receita-base</t>
         </is>
       </c>
       <c r="B7" s="15" t="n">
@@ -4798,47 +4803,47 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>52,0% — praticamente na janela</t>
+          <t>52,0%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Pleito R$ 24,29 mi · 14 anos / 4 carência · preço R$ 82/t</t>
+          <t>Pleito R$ 24,29 mi · 14a · 4 car + 10 amort · receita-base</t>
         </is>
       </c>
       <c r="B8" s="15" t="n">
-        <v>0.4700902764365716</v>
+        <v>0.5732451073480566</v>
       </c>
       <c r="C8" s="28" t="inlineStr">
         <is>
-          <t>PASSA</t>
+          <t>NÃO PASSA</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>47,0% — dentro da janela</t>
+          <t>57,3%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Pleito R$ 24,29 mi · 14a/4c · preço 82 + teto da licença</t>
+          <t>Pleito R$ 24,29 mi · 12a/3c · receita-base (sem condição Mulher)</t>
         </is>
       </c>
       <c r="B9" s="15" t="n">
-        <v>0.3679927983211566</v>
+        <v>0.6386693237419049</v>
       </c>
       <c r="C9" s="28" t="inlineStr">
         <is>
-          <t>PASSA</t>
+          <t>NÃO PASSA</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>36,8% — folga</t>
+          <t>referência</t>
         </is>
       </c>
     </row>
@@ -4852,31 +4857,31 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>14 anos / 4 carência · receita-base</t>
+          <t>14a · 2c+12a · receita-base</t>
         </is>
       </c>
       <c r="B12" s="14" t="n">
-        <v>21855240.32583817</v>
+        <v>24840000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>14 anos / 4 carência · preço R$ 82/t</t>
+          <t>14a · 2c+12a · preço R$ 82/t</t>
         </is>
       </c>
       <c r="B13" s="14" t="n">
-        <v>25506796.63585015</v>
+        <v>28980000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>12 anos / 3 carência · receita-base (referência)</t>
+          <t>14a · 4c+10a · receita-base (comparação)</t>
         </is>
       </c>
       <c r="B14" s="14" t="n">
-        <v>20062332.39691937</v>
+        <v>21855240.32583817</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
Adiciona aba Mix_Produtos: ponderação linha a linha do preço médio
- A: mix real vendido PVV 2025 (8 SKUs, 75.189 t) x preços líquidos → R$ 76,80/t FOB
- B: reconciliação consolidado R$ 116,14 − 36,2% logística → FOB-eq R$ 74,08 → caso-base R$ 68,50 (−7,5%)
- C: mix de projeto do PAE (35% brita ¾ / 25% gravilhão / 40% pó)
- D: teste de estresse do pó (piso R$ 58,89–69,29) + mitigações
- E: produtos da carta consulta x SKUs reais da PVV (veredito: portfólio idêntico)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DqEaERD1LDFtugtNrL73cp
</commit_message>
<xml_diff>
--- a/Viabilidade_CIPREM.xlsx
+++ b/Viabilidade_CIPREM.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Premissas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="DRE_PVV_2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Producao_Receita" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Custos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FNE_SAC" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="DRE_Projetada" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Fluxo_Indicadores" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Capacidade_BNB" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Sensibilidade" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premissas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DRE_PVV_2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mix_Produtos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Producao_Receita" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FNE_SAC" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DRE_Projetada" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fluxo_Indicadores" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacidade_BNB" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensibilidade" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,10 +26,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="#,##0;(#,##0);-"/>
     <numFmt numFmtId="166" formatCode="R$ #,##0;(R$ #,##0);-"/>
+    <numFmt numFmtId="167" formatCode="R$ #,##0.00"/>
+    <numFmt numFmtId="168" formatCode="R$ #,##0"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -122,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -154,6 +157,19 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -519,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -649,12 +665,249 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Mix_Produtos → de onde vem o R$/t: mix real da PVV linha a linha, reconciliação até o caso-base (R$ 68,50) e verificação produto a produto da carta consulta.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CAPACIDADE DE PAGAMENTO — MOTOR OFICIAL BNB (janela 30–50%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Rédito = Receita BRUTA × (1 − custo padrão). Valores calculados no algoritmo VBA real do banco (script da consultoria, validado ao centésimo). Custo padrão proposto: 68,62% (DRE real PVV); tabela indústria: 67,77% — VALIDAR com o analista.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Configuração</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Comprometimento máx.</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Veredito</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Pleito R$ 24,29 mi · 14a · 2 car + 12 amort · receita ultra-conservadora</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="n">
+        <v>0.5095582712098438</v>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>NÃO PASSA</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>51,0% — 1 p.p. fora; fecha com preço R$ 74/t (46,5%), platô antecipado (49,8%) ou 95% (42,0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Pleito R$ 24,29 mi · 14a · 2 car + 12 amort · preço R$ 82/t</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>0.413330734071942</v>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>PASSA</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>41,3% — colchão</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Pleito R$ 24,29 mi · 14a · 2 car + 12 amort · produção 95% da licença</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>0.4195555249059341</v>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>PASSA</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>42,0% — colchão</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Pleito R$ 24,29 mi · 14a · 3 car + 11 amort · receita-base</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>0.5449953606863867</v>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>NÃO PASSA</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>54,5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Pleito R$ 24,29 mi · 14a · 4 car + 10 amort · receita-base</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>0.6010854034324153</v>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>NÃO PASSA</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>60,1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Pleito R$ 24,29 mi · 12a/3c · receita-base (sem condição Mulher)</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>0.6700428550535171</v>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>NÃO PASSA</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>67,0% — referência</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>FINANCIAMENTO MÁXIMO QUE PASSA (≤50%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>14a · 2c+12a · receita-base</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="n">
+        <v>23964142.38999998</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>14a · 2c+12a · preço R$ 82/t</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="n">
+        <v>27958836.32254746</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>14a · 2c+12a · produção 95% da licença</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="n">
+        <v>27660200.76147405</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>14a · 4c+10a · receita-base (comparação)</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="n">
+        <v>21200497.68732259</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Formulas sem cache: o Excel recalcula ao abrir. Nota: valores estáticos (o algoritmo do banco não é replicável em fórmula de planilha). Para recalcular após mudar premissas, rodar o script capacidade_pagamento.py da skill do consultor.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2267,545 +2520,862 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PRODUÇÃO E RECEITA — 12 ANOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 1</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 2</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 3</t>
-        </is>
-      </c>
-      <c r="F3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 4</t>
-        </is>
-      </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 5</t>
-        </is>
-      </c>
-      <c r="H3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 6</t>
-        </is>
-      </c>
-      <c r="I3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 7</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 8</t>
-        </is>
-      </c>
-      <c r="K3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 9</t>
-        </is>
-      </c>
-      <c r="L3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 10</t>
-        </is>
-      </c>
-      <c r="M3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 11</t>
-        </is>
-      </c>
-      <c r="N3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 12</t>
-        </is>
-      </c>
-      <c r="O3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 13</t>
-        </is>
-      </c>
-      <c r="P3" s="13" t="inlineStr">
-        <is>
-          <t>Ano 14</t>
+          <t>MIX DE PRODUTOS — DE ONDE VEM O PREÇO MÉDIO POR TONELADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>A britagem gera vários produtos com preços muito diferentes; o modelo NÃO usa preço de um produto único: usa a média ponderada do mix real vendido pela pedreira-modelo (PVV) em 2025, reconciliada abaixo. Azul = dado de documento · preto = fórmula · verde = link entre abas.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Vendas (t)</t>
-        </is>
-      </c>
-      <c r="C4" s="18">
-        <f>Premissas!C$38</f>
-        <v/>
-      </c>
-      <c r="D4" s="18">
-        <f>Premissas!D$38</f>
-        <v/>
-      </c>
-      <c r="E4" s="18">
-        <f>Premissas!E$38</f>
-        <v/>
-      </c>
-      <c r="F4" s="18">
-        <f>Premissas!F$38</f>
-        <v/>
-      </c>
-      <c r="G4" s="18">
-        <f>Premissas!G$38</f>
-        <v/>
-      </c>
-      <c r="H4" s="18">
-        <f>Premissas!H$38</f>
-        <v/>
-      </c>
-      <c r="I4" s="18">
-        <f>Premissas!I$38</f>
-        <v/>
-      </c>
-      <c r="J4" s="18">
-        <f>Premissas!J$38</f>
-        <v/>
-      </c>
-      <c r="K4" s="18">
-        <f>Premissas!K$38</f>
-        <v/>
-      </c>
-      <c r="L4" s="18">
-        <f>Premissas!L$38</f>
-        <v/>
-      </c>
-      <c r="M4" s="18">
-        <f>Premissas!M$38</f>
-        <v/>
-      </c>
-      <c r="N4" s="18">
-        <f>Premissas!N$38</f>
-        <v/>
-      </c>
-      <c r="O4" s="18">
-        <f>Premissas!O$38</f>
-        <v/>
-      </c>
-      <c r="P4" s="18">
-        <f>Premissas!P$38</f>
-        <v/>
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>A · O QUE A PEDREIRA-MODELO (PVV) VENDEU EM 2025 — na pedreira, FOB (sem frete)</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Vendas CIF (t)</t>
-        </is>
-      </c>
-      <c r="C5" s="18">
-        <f>MIN(C4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
-      </c>
-      <c r="D5" s="18">
-        <f>MIN(D4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
-      </c>
-      <c r="E5" s="18">
-        <f>MIN(E4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
-      </c>
-      <c r="F5" s="18">
-        <f>MIN(F4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
-      </c>
-      <c r="G5" s="18">
-        <f>MIN(G4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
-      </c>
-      <c r="H5" s="18">
-        <f>MIN(H4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
-      </c>
-      <c r="I5" s="18">
-        <f>MIN(I4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
-      </c>
-      <c r="J5" s="18">
-        <f>MIN(J4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
-      </c>
-      <c r="K5" s="18">
-        <f>MIN(K4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
-      </c>
-      <c r="L5" s="18">
-        <f>MIN(L4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
-      </c>
-      <c r="M5" s="18">
-        <f>MIN(M4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
-      </c>
-      <c r="N5" s="18">
-        <f>MIN(N4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
-      </c>
-      <c r="O5" s="18">
-        <f>MIN(O4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
-      </c>
-      <c r="P5" s="18">
-        <f>MIN(P4*Premissas!$B$13,Premissas!$B$14)</f>
-        <v/>
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>t vendidas</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>% do mix</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Preço tabela (R$/t)</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Desconto médio</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>Preço líquido (R$/t)</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>Receita FOB (R$)</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Receita FOB (R$)</t>
-        </is>
-      </c>
-      <c r="C6" s="19">
-        <f>C4*Premissas!$B$10</f>
-        <v/>
-      </c>
-      <c r="D6" s="19">
-        <f>D4*Premissas!$B$10</f>
-        <v/>
-      </c>
-      <c r="E6" s="19">
-        <f>E4*Premissas!$B$10</f>
-        <v/>
-      </c>
-      <c r="F6" s="19">
-        <f>F4*Premissas!$B$10</f>
-        <v/>
-      </c>
-      <c r="G6" s="19">
-        <f>G4*Premissas!$B$10</f>
-        <v/>
-      </c>
-      <c r="H6" s="19">
-        <f>H4*Premissas!$B$10</f>
-        <v/>
-      </c>
-      <c r="I6" s="19">
-        <f>I4*Premissas!$B$10</f>
-        <v/>
-      </c>
-      <c r="J6" s="19">
-        <f>J4*Premissas!$B$10</f>
-        <v/>
-      </c>
-      <c r="K6" s="19">
-        <f>K4*Premissas!$B$10</f>
-        <v/>
-      </c>
-      <c r="L6" s="19">
-        <f>L4*Premissas!$B$10</f>
-        <v/>
-      </c>
-      <c r="M6" s="19">
-        <f>M4*Premissas!$B$10</f>
-        <v/>
-      </c>
-      <c r="N6" s="19">
-        <f>N4*Premissas!$B$10</f>
-        <v/>
-      </c>
-      <c r="O6" s="19">
-        <f>O4*Premissas!$B$10</f>
-        <v/>
-      </c>
-      <c r="P6" s="19">
-        <f>P4*Premissas!$B$10</f>
-        <v/>
+          <t>BRITA 1</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>24949.64</v>
+      </c>
+      <c r="C6" s="15">
+        <f>B6/$B$14</f>
+        <v/>
+      </c>
+      <c r="D6" s="30" t="n">
+        <v>98</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F6" s="31">
+        <f>D6*(1-E6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="32">
+        <f>B6*F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>na carta CIPREM: brita 1</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Receita de frete CIF (R$)</t>
-        </is>
-      </c>
-      <c r="C7" s="19">
-        <f>C5*Premissas!$B$15</f>
-        <v/>
-      </c>
-      <c r="D7" s="19">
-        <f>D5*Premissas!$B$15</f>
-        <v/>
-      </c>
-      <c r="E7" s="19">
-        <f>E5*Premissas!$B$15</f>
-        <v/>
-      </c>
-      <c r="F7" s="19">
-        <f>F5*Premissas!$B$15</f>
-        <v/>
-      </c>
-      <c r="G7" s="19">
-        <f>G5*Premissas!$B$15</f>
-        <v/>
-      </c>
-      <c r="H7" s="19">
-        <f>H5*Premissas!$B$15</f>
-        <v/>
-      </c>
-      <c r="I7" s="19">
-        <f>I5*Premissas!$B$15</f>
-        <v/>
-      </c>
-      <c r="J7" s="19">
-        <f>J5*Premissas!$B$15</f>
-        <v/>
-      </c>
-      <c r="K7" s="19">
-        <f>K5*Premissas!$B$15</f>
-        <v/>
-      </c>
-      <c r="L7" s="19">
-        <f>L5*Premissas!$B$15</f>
-        <v/>
-      </c>
-      <c r="M7" s="19">
-        <f>M5*Premissas!$B$15</f>
-        <v/>
-      </c>
-      <c r="N7" s="19">
-        <f>N5*Premissas!$B$15</f>
-        <v/>
-      </c>
-      <c r="O7" s="19">
-        <f>O5*Premissas!$B$15</f>
-        <v/>
-      </c>
-      <c r="P7" s="19">
-        <f>P5*Premissas!$B$15</f>
-        <v/>
+          <t>PÓ DE PEDRA</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>16312.55</v>
+      </c>
+      <c r="C7" s="15">
+        <f>B7/$B$14</f>
+        <v/>
+      </c>
+      <c r="D7" s="30" t="n">
+        <v>25</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F7" s="31">
+        <f>D7*(1-E7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="32">
+        <f>B7*F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>na carta: pó de pedra — 22% do mix na pedreira; sobe a 29% no consolidado</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>RECEITA BRUTA (R$)</t>
-        </is>
-      </c>
-      <c r="C8" s="14">
-        <f>C6+C7</f>
-        <v/>
-      </c>
-      <c r="D8" s="14">
-        <f>D6+D7</f>
-        <v/>
-      </c>
-      <c r="E8" s="14">
-        <f>E6+E7</f>
-        <v/>
-      </c>
-      <c r="F8" s="14">
-        <f>F6+F7</f>
-        <v/>
-      </c>
-      <c r="G8" s="14">
-        <f>G6+G7</f>
-        <v/>
-      </c>
-      <c r="H8" s="14">
-        <f>H6+H7</f>
-        <v/>
-      </c>
-      <c r="I8" s="14">
-        <f>I6+I7</f>
-        <v/>
-      </c>
-      <c r="J8" s="14">
-        <f>J6+J7</f>
-        <v/>
-      </c>
-      <c r="K8" s="14">
-        <f>K6+K7</f>
-        <v/>
-      </c>
-      <c r="L8" s="14">
-        <f>L6+L7</f>
-        <v/>
-      </c>
-      <c r="M8" s="14">
-        <f>M6+M7</f>
-        <v/>
-      </c>
-      <c r="N8" s="14">
-        <f>N6+N7</f>
-        <v/>
-      </c>
-      <c r="O8" s="14">
-        <f>O6+O7</f>
-        <v/>
-      </c>
-      <c r="P8" s="14">
-        <f>P6+P7</f>
-        <v/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>BRITA 0</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>13608.91</v>
+      </c>
+      <c r="C8" s="15">
+        <f>B8/$B$14</f>
+        <v/>
+      </c>
+      <c r="D8" s="30" t="n">
+        <v>120</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F8" s="31">
+        <f>D8*(1-E8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="32">
+        <f>B8*F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>na carta: brita 0</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>(–) Deduções (R$)</t>
-        </is>
-      </c>
-      <c r="C9" s="19">
-        <f>-C8*Premissas!$B$17</f>
-        <v/>
-      </c>
-      <c r="D9" s="19">
-        <f>-D8*Premissas!$B$17</f>
-        <v/>
-      </c>
-      <c r="E9" s="19">
-        <f>-E8*Premissas!$B$17</f>
-        <v/>
-      </c>
-      <c r="F9" s="19">
-        <f>-F8*Premissas!$B$17</f>
-        <v/>
-      </c>
-      <c r="G9" s="19">
-        <f>-G8*Premissas!$B$17</f>
-        <v/>
-      </c>
-      <c r="H9" s="19">
-        <f>-H8*Premissas!$B$17</f>
-        <v/>
-      </c>
-      <c r="I9" s="19">
-        <f>-I8*Premissas!$B$17</f>
-        <v/>
-      </c>
-      <c r="J9" s="19">
-        <f>-J8*Premissas!$B$17</f>
-        <v/>
-      </c>
-      <c r="K9" s="19">
-        <f>-K8*Premissas!$B$17</f>
-        <v/>
-      </c>
-      <c r="L9" s="19">
-        <f>-L8*Premissas!$B$17</f>
-        <v/>
-      </c>
-      <c r="M9" s="19">
-        <f>-M8*Premissas!$B$17</f>
-        <v/>
-      </c>
-      <c r="N9" s="19">
-        <f>-N8*Premissas!$B$17</f>
-        <v/>
-      </c>
-      <c r="O9" s="19">
-        <f>-O8*Premissas!$B$17</f>
-        <v/>
-      </c>
-      <c r="P9" s="19">
-        <f>-P8*Premissas!$B$17</f>
-        <v/>
+          <t>PULMÃO (rachão)</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>6640.27</v>
+      </c>
+      <c r="C9" s="15">
+        <f>B9/$B$14</f>
+        <v/>
+      </c>
+      <c r="D9" s="30" t="n">
+        <v>85</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F9" s="31">
+        <f>D9*(1-E9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="32">
+        <f>B9*F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>não listado na carta; PAE prevê "sob demanda"</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>RECEITA LÍQUIDA (R$)</t>
-        </is>
-      </c>
-      <c r="C10" s="14">
-        <f>C8+C9</f>
-        <v/>
-      </c>
-      <c r="D10" s="14">
-        <f>D8+D9</f>
-        <v/>
-      </c>
-      <c r="E10" s="14">
-        <f>E8+E9</f>
-        <v/>
-      </c>
-      <c r="F10" s="14">
-        <f>F8+F9</f>
-        <v/>
-      </c>
-      <c r="G10" s="14">
-        <f>G8+G9</f>
-        <v/>
-      </c>
-      <c r="H10" s="14">
-        <f>H8+H9</f>
-        <v/>
-      </c>
-      <c r="I10" s="14">
-        <f>I8+I9</f>
-        <v/>
-      </c>
-      <c r="J10" s="14">
-        <f>J8+J9</f>
-        <v/>
-      </c>
-      <c r="K10" s="14">
-        <f>K8+K9</f>
-        <v/>
-      </c>
-      <c r="L10" s="14">
-        <f>L8+L9</f>
-        <v/>
-      </c>
-      <c r="M10" s="14">
-        <f>M8+M9</f>
-        <v/>
-      </c>
-      <c r="N10" s="14">
-        <f>N8+N9</f>
-        <v/>
-      </c>
-      <c r="O10" s="14">
-        <f>O8+O9</f>
-        <v/>
-      </c>
-      <c r="P10" s="14">
-        <f>P8+P9</f>
-        <v/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>BRITA GRADUADA (BGS)</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>4562.89</v>
+      </c>
+      <c r="C10" s="15">
+        <f>B10/$B$14</f>
+        <v/>
+      </c>
+      <c r="D10" s="30" t="n">
+        <v>85</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="F10" s="31">
+        <f>D10*(1-E10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="32">
+        <f>B10*F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>na carta: BGS/solo-brita — mistura de pó + britas</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>PEDRISCO</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>4279.26</v>
+      </c>
+      <c r="C11" s="15">
+        <f>B11/$B$14</f>
+        <v/>
+      </c>
+      <c r="D11" s="30" t="n">
+        <v>80</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F11" s="31">
+        <f>D11*(1-E11)</f>
+        <v/>
+      </c>
+      <c r="G11" s="32">
+        <f>B11*F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>na carta: gravilinha (nome regional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>BRITA 2</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>4253.52</v>
+      </c>
+      <c r="C12" s="15">
+        <f>B12/$B$14</f>
+        <v/>
+      </c>
+      <c r="D12" s="30" t="n">
+        <v>98</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F12" s="31">
+        <f>D12*(1-E12)</f>
+        <v/>
+      </c>
+      <c r="G12" s="32">
+        <f>B12*F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>na carta: brita 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>MARROADA</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>582.2</v>
+      </c>
+      <c r="C13" s="15">
+        <f>B13/$B$14</f>
+        <v/>
+      </c>
+      <c r="D13" s="30" t="n">
+        <v>87</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F13" s="31">
+        <f>D13*(1-E13)</f>
+        <v/>
+      </c>
+      <c r="G13" s="32">
+        <f>B13*F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>não listada na carta; venda eventual</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>TOTAL / PREÇO MÉDIO PONDERADO FOB PEDREIRA</t>
+        </is>
+      </c>
+      <c r="B14" s="33">
+        <f>SUM(B6:B13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="34">
+        <f>SUM(C6:C13)</f>
+        <v/>
+      </c>
+      <c r="F14" s="35">
+        <f>G14/B14</f>
+        <v/>
+      </c>
+      <c r="G14" s="36">
+        <f>SUM(G6:G13)</f>
+        <v/>
+      </c>
+      <c r="H14" s="37" t="inlineStr">
+        <is>
+          <t>≈ R$ 76,80/t — nenhum produto isolado: é a tonelada média do mix inteiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>B · DA OPERAÇÃO REAL AO PREÇO DO MODELO — RECONCILIAÇÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Preço médio FOB pedreira (mix real, seção A)</t>
+        </is>
+      </c>
+      <c r="F17" s="31">
+        <f>F14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Preço médio realizado consolidado 2025 (pedreira + filiais Porto Seguro e Trancoso)</t>
+        </is>
+      </c>
+      <c r="F18" s="30" t="n">
+        <v>116.135488216766</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>ver aba DRE_PVV_2025 — inclui preços de varejo das filiais e a logística até elas</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Logística/estrutura de filiais embutida no consolidado</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0.3621264721735005</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>FOB-EQUIVALENTE (consolidado × (1 − logística)) — o número-âncora</t>
+        </is>
+      </c>
+      <c r="F20" s="35">
+        <f>F18*(1-F19)</f>
+        <v/>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>≈ R$ 74,08/t — o que a tonelada média rende tirando o custo de levá-la às filiais</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>PREÇO DO CASO-BASE DO MODELO (aba Premissas)</t>
+        </is>
+      </c>
+      <c r="F21" s="30" t="n">
+        <v>68.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Margem de prudência adotada sobre o FOB-equivalente</t>
+        </is>
+      </c>
+      <c r="F22" s="15">
+        <f>1-F21/F20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Sensibilidade (aba Sensibilidade): a R$ 74/t o comprometimento cai a 46,5%; a R$ 82/t, a 41,3%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Nas filiais o pó de pedra NÃO sai a R$ 25: tabela Porto Seguro R$ 56,71/t · Trancoso R$ 64,47/t.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>C · MIX DE PROJETO DA CIPREM — tabela de produtos do PAE (planta a 20.000 t/mês)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Produto (nome no PAE)</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Equivalente comercial</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>Faixa</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>% da produção</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>t/mês</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Brita 19 mm (¾")</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>brita 1</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>19–12,5 mm</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E28" s="28">
+        <f>D28*20000</f>
+        <v/>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>produto de maior giro</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Brita 12,5 mm (½") — "Gravilhão"</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>brita 0 / gravilinha</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>12,5–4,8 mm</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E29" s="28">
+        <f>D29*20000</f>
+        <v/>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Brita 4,8 mm (pó de pedra)</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>pó de pedra</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>&lt; 4,8 mm</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E30" s="28">
+        <f>D30*20000</f>
+        <v/>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>fração crítica — ver seção D</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Brita 76/38 mm (3"/2") e rachão</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>brita 2 / rachão</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>sob demanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Brita graduada (BGS)</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>BGS/solo-brita</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>recombinação de pó + britas (não é massa nova)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Fonte: PAE CIPREM, parte 2 — "Produtos do processo de britagem": 7.000 + 5.000 + 8.000 = 20.000 t/mês (35% + 25% + 40%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="29" t="inlineStr">
+        <is>
+          <t>D · TESTE DE ESTRESSE DO MIX — e se o pó só valer o preço mínimo?</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Piso: mix de projeto (35/25/40), fração ½" valendo como PEDRISCO e pó a tabela mínima da pedreira</t>
+        </is>
+      </c>
+      <c r="F36" s="31">
+        <f>0.35*F6+0.25*F11+0.40*F7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Mesmo piso, com a fração ½" valendo como BRITA 0</t>
+        </is>
+      </c>
+      <c r="F37" s="31">
+        <f>0.35*F6+0.25*F8+0.40*F7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Leitura: o caso-base (R$ 68,50) está dentro da banda do piso estressado (F36–F37) e ABAIXO do realizado da operação gêmea (R$ 74–77).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Mitigações que elevam a média de volta: pó misturado em BGS (vende a R$ 85/t) · câmara F-Sand do HP350e (converte fina em areia de brita) · consumo cativo (premoldados da CIPREM + Concreto Britaki) · nas filiais o pó já realiza R$ 57–64/t.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="29" t="inlineStr">
+        <is>
+          <t>E · PRODUTOS DA CARTA CONSULTA × O QUE A PVV REALMENTE VENDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>Produto na carta consulta (CIPREM)</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>PVV vende?</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>SKU na PVV</t>
+        </is>
+      </c>
+      <c r="H42" s="13" t="inlineStr">
+        <is>
+          <t>Observação</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>brita 0</t>
+        </is>
+      </c>
+      <c r="B43" s="38" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>BRITA 0</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>mesmo produto</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>brita 1</t>
+        </is>
+      </c>
+      <c r="B44" s="38" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>BRITA 1</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>mesmo produto — maior giro da PVV (31% do vendido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>brita 2</t>
+        </is>
+      </c>
+      <c r="B45" s="38" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>BRITA 2</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>PAE produz "sob demanda" (4% do vendido na PVV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>gravilinha</t>
+        </is>
+      </c>
+      <c r="B46" s="38" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>PEDRISCO</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>mesmo produto, nome regional diferente</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>pó de pedra</t>
+        </is>
+      </c>
+      <c r="B47" s="38" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>PÓ</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>mesma fração; na PVV é 29% do vendido consolidado</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>BGS/solo-brita</t>
+        </is>
+      </c>
+      <c r="B48" s="38" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>BRITA GRADUADA</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>mesma mistura (pó + britas), nome diferente</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>— (não listados na carta)</t>
+        </is>
+      </c>
+      <c r="B49" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>MARROADA · PULMÃO/RACHÃO</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>a PVV vende e o PAE prevê "sob demanda" — upside não contado no modelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="39" t="inlineStr">
+        <is>
+          <t>VEREDITO: o portfólio da carta é o mesmo que a pedreira-modelo pratica há anos — só muda nomenclatura regional (gravilinha=pedrisco; BGS=brita graduada). Nenhum produto da carta é sem precedente real no grupo.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2843,7 +3413,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CUSTOS E DESPESAS — 12 ANOS</t>
+          <t>PRODUÇÃO E RECEITA — 12 ANOS</t>
         </is>
       </c>
     </row>
@@ -2922,441 +3492,441 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Custo variável de produção (R$)</t>
-        </is>
-      </c>
-      <c r="C4" s="19">
-        <f>Producao_Receita!C4*Premissas!C$21</f>
-        <v/>
-      </c>
-      <c r="D4" s="19">
-        <f>Producao_Receita!D4*Premissas!D$21</f>
-        <v/>
-      </c>
-      <c r="E4" s="19">
-        <f>Producao_Receita!E4*Premissas!E$21</f>
-        <v/>
-      </c>
-      <c r="F4" s="19">
-        <f>Producao_Receita!F4*Premissas!F$21</f>
-        <v/>
-      </c>
-      <c r="G4" s="19">
-        <f>Producao_Receita!G4*Premissas!G$21</f>
-        <v/>
-      </c>
-      <c r="H4" s="19">
-        <f>Producao_Receita!H4*Premissas!H$21</f>
-        <v/>
-      </c>
-      <c r="I4" s="19">
-        <f>Producao_Receita!I4*Premissas!I$21</f>
-        <v/>
-      </c>
-      <c r="J4" s="19">
-        <f>Producao_Receita!J4*Premissas!J$21</f>
-        <v/>
-      </c>
-      <c r="K4" s="19">
-        <f>Producao_Receita!K4*Premissas!K$21</f>
-        <v/>
-      </c>
-      <c r="L4" s="19">
-        <f>Producao_Receita!L4*Premissas!L$21</f>
-        <v/>
-      </c>
-      <c r="M4" s="19">
-        <f>Producao_Receita!M4*Premissas!M$21</f>
-        <v/>
-      </c>
-      <c r="N4" s="19">
-        <f>Producao_Receita!N4*Premissas!N$21</f>
-        <v/>
-      </c>
-      <c r="O4" s="19">
-        <f>Producao_Receita!O4*Premissas!O$21</f>
-        <v/>
-      </c>
-      <c r="P4" s="19">
-        <f>Producao_Receita!P4*Premissas!P$21</f>
+          <t>Vendas (t)</t>
+        </is>
+      </c>
+      <c r="C4" s="18">
+        <f>Premissas!C$38</f>
+        <v/>
+      </c>
+      <c r="D4" s="18">
+        <f>Premissas!D$38</f>
+        <v/>
+      </c>
+      <c r="E4" s="18">
+        <f>Premissas!E$38</f>
+        <v/>
+      </c>
+      <c r="F4" s="18">
+        <f>Premissas!F$38</f>
+        <v/>
+      </c>
+      <c r="G4" s="18">
+        <f>Premissas!G$38</f>
+        <v/>
+      </c>
+      <c r="H4" s="18">
+        <f>Premissas!H$38</f>
+        <v/>
+      </c>
+      <c r="I4" s="18">
+        <f>Premissas!I$38</f>
+        <v/>
+      </c>
+      <c r="J4" s="18">
+        <f>Premissas!J$38</f>
+        <v/>
+      </c>
+      <c r="K4" s="18">
+        <f>Premissas!K$38</f>
+        <v/>
+      </c>
+      <c r="L4" s="18">
+        <f>Premissas!L$38</f>
+        <v/>
+      </c>
+      <c r="M4" s="18">
+        <f>Premissas!M$38</f>
+        <v/>
+      </c>
+      <c r="N4" s="18">
+        <f>Premissas!N$38</f>
+        <v/>
+      </c>
+      <c r="O4" s="18">
+        <f>Premissas!O$38</f>
+        <v/>
+      </c>
+      <c r="P4" s="18">
+        <f>Premissas!P$38</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Custo do frete próprio (R$)</t>
-        </is>
-      </c>
-      <c r="C5" s="19">
-        <f>Producao_Receita!C7*Premissas!$B$16</f>
-        <v/>
-      </c>
-      <c r="D5" s="19">
-        <f>Producao_Receita!D7*Premissas!$B$16</f>
-        <v/>
-      </c>
-      <c r="E5" s="19">
-        <f>Producao_Receita!E7*Premissas!$B$16</f>
-        <v/>
-      </c>
-      <c r="F5" s="19">
-        <f>Producao_Receita!F7*Premissas!$B$16</f>
-        <v/>
-      </c>
-      <c r="G5" s="19">
-        <f>Producao_Receita!G7*Premissas!$B$16</f>
-        <v/>
-      </c>
-      <c r="H5" s="19">
-        <f>Producao_Receita!H7*Premissas!$B$16</f>
-        <v/>
-      </c>
-      <c r="I5" s="19">
-        <f>Producao_Receita!I7*Premissas!$B$16</f>
-        <v/>
-      </c>
-      <c r="J5" s="19">
-        <f>Producao_Receita!J7*Premissas!$B$16</f>
-        <v/>
-      </c>
-      <c r="K5" s="19">
-        <f>Producao_Receita!K7*Premissas!$B$16</f>
-        <v/>
-      </c>
-      <c r="L5" s="19">
-        <f>Producao_Receita!L7*Premissas!$B$16</f>
-        <v/>
-      </c>
-      <c r="M5" s="19">
-        <f>Producao_Receita!M7*Premissas!$B$16</f>
-        <v/>
-      </c>
-      <c r="N5" s="19">
-        <f>Producao_Receita!N7*Premissas!$B$16</f>
-        <v/>
-      </c>
-      <c r="O5" s="19">
-        <f>Producao_Receita!O7*Premissas!$B$16</f>
-        <v/>
-      </c>
-      <c r="P5" s="19">
-        <f>Producao_Receita!P7*Premissas!$B$16</f>
+          <t>Vendas CIF (t)</t>
+        </is>
+      </c>
+      <c r="C5" s="18">
+        <f>MIN(C4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="D5" s="18">
+        <f>MIN(D4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="E5" s="18">
+        <f>MIN(E4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="F5" s="18">
+        <f>MIN(F4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="G5" s="18">
+        <f>MIN(G4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="H5" s="18">
+        <f>MIN(H4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="I5" s="18">
+        <f>MIN(I4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="J5" s="18">
+        <f>MIN(J4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="K5" s="18">
+        <f>MIN(K4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="L5" s="18">
+        <f>MIN(L4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="M5" s="18">
+        <f>MIN(M4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="N5" s="18">
+        <f>MIN(N4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="O5" s="18">
+        <f>MIN(O4*Premissas!$B$13,Premissas!$B$14)</f>
+        <v/>
+      </c>
+      <c r="P5" s="18">
+        <f>MIN(P4*Premissas!$B$13,Premissas!$B$14)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CFEM (R$)</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Receita FOB (R$)</t>
         </is>
       </c>
       <c r="C6" s="19">
-        <f>Producao_Receita!C8*Premissas!$B$18</f>
+        <f>C4*Premissas!$B$10</f>
         <v/>
       </c>
       <c r="D6" s="19">
-        <f>Producao_Receita!D8*Premissas!$B$18</f>
+        <f>D4*Premissas!$B$10</f>
         <v/>
       </c>
       <c r="E6" s="19">
-        <f>Producao_Receita!E8*Premissas!$B$18</f>
+        <f>E4*Premissas!$B$10</f>
         <v/>
       </c>
       <c r="F6" s="19">
-        <f>Producao_Receita!F8*Premissas!$B$18</f>
+        <f>F4*Premissas!$B$10</f>
         <v/>
       </c>
       <c r="G6" s="19">
-        <f>Producao_Receita!G8*Premissas!$B$18</f>
+        <f>G4*Premissas!$B$10</f>
         <v/>
       </c>
       <c r="H6" s="19">
-        <f>Producao_Receita!H8*Premissas!$B$18</f>
+        <f>H4*Premissas!$B$10</f>
         <v/>
       </c>
       <c r="I6" s="19">
-        <f>Producao_Receita!I8*Premissas!$B$18</f>
+        <f>I4*Premissas!$B$10</f>
         <v/>
       </c>
       <c r="J6" s="19">
-        <f>Producao_Receita!J8*Premissas!$B$18</f>
+        <f>J4*Premissas!$B$10</f>
         <v/>
       </c>
       <c r="K6" s="19">
-        <f>Producao_Receita!K8*Premissas!$B$18</f>
+        <f>K4*Premissas!$B$10</f>
         <v/>
       </c>
       <c r="L6" s="19">
-        <f>Producao_Receita!L8*Premissas!$B$18</f>
+        <f>L4*Premissas!$B$10</f>
         <v/>
       </c>
       <c r="M6" s="19">
-        <f>Producao_Receita!M8*Premissas!$B$18</f>
+        <f>M4*Premissas!$B$10</f>
         <v/>
       </c>
       <c r="N6" s="19">
-        <f>Producao_Receita!N8*Premissas!$B$18</f>
+        <f>N4*Premissas!$B$10</f>
         <v/>
       </c>
       <c r="O6" s="19">
-        <f>Producao_Receita!O8*Premissas!$B$18</f>
+        <f>O4*Premissas!$B$10</f>
         <v/>
       </c>
       <c r="P6" s="19">
-        <f>Producao_Receita!P8*Premissas!$B$18</f>
+        <f>P4*Premissas!$B$10</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Custos fixos de produção (R$)</t>
+          <t>Receita de frete CIF (R$)</t>
         </is>
       </c>
       <c r="C7" s="19">
-        <f>Premissas!C$22</f>
+        <f>C5*Premissas!$B$15</f>
         <v/>
       </c>
       <c r="D7" s="19">
-        <f>Premissas!D$22</f>
+        <f>D5*Premissas!$B$15</f>
         <v/>
       </c>
       <c r="E7" s="19">
-        <f>Premissas!E$22</f>
+        <f>E5*Premissas!$B$15</f>
         <v/>
       </c>
       <c r="F7" s="19">
-        <f>Premissas!F$22</f>
+        <f>F5*Premissas!$B$15</f>
         <v/>
       </c>
       <c r="G7" s="19">
-        <f>Premissas!G$22</f>
+        <f>G5*Premissas!$B$15</f>
         <v/>
       </c>
       <c r="H7" s="19">
-        <f>Premissas!H$22</f>
+        <f>H5*Premissas!$B$15</f>
         <v/>
       </c>
       <c r="I7" s="19">
-        <f>Premissas!I$22</f>
+        <f>I5*Premissas!$B$15</f>
         <v/>
       </c>
       <c r="J7" s="19">
-        <f>Premissas!J$22</f>
+        <f>J5*Premissas!$B$15</f>
         <v/>
       </c>
       <c r="K7" s="19">
-        <f>Premissas!K$22</f>
+        <f>K5*Premissas!$B$15</f>
         <v/>
       </c>
       <c r="L7" s="19">
-        <f>Premissas!L$22</f>
+        <f>L5*Premissas!$B$15</f>
         <v/>
       </c>
       <c r="M7" s="19">
-        <f>Premissas!M$22</f>
+        <f>M5*Premissas!$B$15</f>
         <v/>
       </c>
       <c r="N7" s="19">
-        <f>Premissas!N$22</f>
+        <f>N5*Premissas!$B$15</f>
         <v/>
       </c>
       <c r="O7" s="19">
-        <f>Premissas!O$22</f>
+        <f>O5*Premissas!$B$15</f>
         <v/>
       </c>
       <c r="P7" s="19">
-        <f>Premissas!P$22</f>
+        <f>P5*Premissas!$B$15</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Despesas adm/com/trib (R$)</t>
-        </is>
-      </c>
-      <c r="C8" s="19">
-        <f>Premissas!C$23</f>
-        <v/>
-      </c>
-      <c r="D8" s="19">
-        <f>Premissas!D$23</f>
-        <v/>
-      </c>
-      <c r="E8" s="19">
-        <f>Premissas!E$23</f>
-        <v/>
-      </c>
-      <c r="F8" s="19">
-        <f>Premissas!F$23</f>
-        <v/>
-      </c>
-      <c r="G8" s="19">
-        <f>Premissas!G$23</f>
-        <v/>
-      </c>
-      <c r="H8" s="19">
-        <f>Premissas!H$23</f>
-        <v/>
-      </c>
-      <c r="I8" s="19">
-        <f>Premissas!I$23</f>
-        <v/>
-      </c>
-      <c r="J8" s="19">
-        <f>Premissas!J$23</f>
-        <v/>
-      </c>
-      <c r="K8" s="19">
-        <f>Premissas!K$23</f>
-        <v/>
-      </c>
-      <c r="L8" s="19">
-        <f>Premissas!L$23</f>
-        <v/>
-      </c>
-      <c r="M8" s="19">
-        <f>Premissas!M$23</f>
-        <v/>
-      </c>
-      <c r="N8" s="19">
-        <f>Premissas!N$23</f>
-        <v/>
-      </c>
-      <c r="O8" s="19">
-        <f>Premissas!O$23</f>
-        <v/>
-      </c>
-      <c r="P8" s="19">
-        <f>Premissas!P$23</f>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>RECEITA BRUTA (R$)</t>
+        </is>
+      </c>
+      <c r="C8" s="14">
+        <f>C6+C7</f>
+        <v/>
+      </c>
+      <c r="D8" s="14">
+        <f>D6+D7</f>
+        <v/>
+      </c>
+      <c r="E8" s="14">
+        <f>E6+E7</f>
+        <v/>
+      </c>
+      <c r="F8" s="14">
+        <f>F6+F7</f>
+        <v/>
+      </c>
+      <c r="G8" s="14">
+        <f>G6+G7</f>
+        <v/>
+      </c>
+      <c r="H8" s="14">
+        <f>H6+H7</f>
+        <v/>
+      </c>
+      <c r="I8" s="14">
+        <f>I6+I7</f>
+        <v/>
+      </c>
+      <c r="J8" s="14">
+        <f>J6+J7</f>
+        <v/>
+      </c>
+      <c r="K8" s="14">
+        <f>K6+K7</f>
+        <v/>
+      </c>
+      <c r="L8" s="14">
+        <f>L6+L7</f>
+        <v/>
+      </c>
+      <c r="M8" s="14">
+        <f>M6+M7</f>
+        <v/>
+      </c>
+      <c r="N8" s="14">
+        <f>N6+N7</f>
+        <v/>
+      </c>
+      <c r="O8" s="14">
+        <f>O6+O7</f>
+        <v/>
+      </c>
+      <c r="P8" s="14">
+        <f>P6+P7</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Custeio grupo (R$)</t>
+          <t>(–) Deduções (R$)</t>
         </is>
       </c>
       <c r="C9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-C8*Premissas!$B$17</f>
         <v/>
       </c>
       <c r="D9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-D8*Premissas!$B$17</f>
         <v/>
       </c>
       <c r="E9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-E8*Premissas!$B$17</f>
         <v/>
       </c>
       <c r="F9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-F8*Premissas!$B$17</f>
         <v/>
       </c>
       <c r="G9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-G8*Premissas!$B$17</f>
         <v/>
       </c>
       <c r="H9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-H8*Premissas!$B$17</f>
         <v/>
       </c>
       <c r="I9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-I8*Premissas!$B$17</f>
         <v/>
       </c>
       <c r="J9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-J8*Premissas!$B$17</f>
         <v/>
       </c>
       <c r="K9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-K8*Premissas!$B$17</f>
         <v/>
       </c>
       <c r="L9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-L8*Premissas!$B$17</f>
         <v/>
       </c>
       <c r="M9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-M8*Premissas!$B$17</f>
         <v/>
       </c>
       <c r="N9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-N8*Premissas!$B$17</f>
         <v/>
       </c>
       <c r="O9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-O8*Premissas!$B$17</f>
         <v/>
       </c>
       <c r="P9" s="19">
-        <f>Premissas!$B$24</f>
+        <f>-P8*Premissas!$B$17</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>TOTAL CUSTOS E DESPESAS (R$)</t>
-        </is>
-      </c>
-      <c r="C10" s="19">
-        <f>SUM(C4:C9)</f>
-        <v/>
-      </c>
-      <c r="D10" s="19">
-        <f>SUM(D4:D9)</f>
-        <v/>
-      </c>
-      <c r="E10" s="19">
-        <f>SUM(E4:E9)</f>
-        <v/>
-      </c>
-      <c r="F10" s="19">
-        <f>SUM(F4:F9)</f>
-        <v/>
-      </c>
-      <c r="G10" s="19">
-        <f>SUM(G4:G9)</f>
-        <v/>
-      </c>
-      <c r="H10" s="19">
-        <f>SUM(H4:H9)</f>
-        <v/>
-      </c>
-      <c r="I10" s="19">
-        <f>SUM(I4:I9)</f>
-        <v/>
-      </c>
-      <c r="J10" s="19">
-        <f>SUM(J4:J9)</f>
-        <v/>
-      </c>
-      <c r="K10" s="19">
-        <f>SUM(K4:K9)</f>
-        <v/>
-      </c>
-      <c r="L10" s="19">
-        <f>SUM(L4:L9)</f>
-        <v/>
-      </c>
-      <c r="M10" s="19">
-        <f>SUM(M4:M9)</f>
-        <v/>
-      </c>
-      <c r="N10" s="19">
-        <f>SUM(N4:N9)</f>
-        <v/>
-      </c>
-      <c r="O10" s="19">
-        <f>SUM(O4:O9)</f>
-        <v/>
-      </c>
-      <c r="P10" s="19">
-        <f>SUM(P4:P9)</f>
+          <t>RECEITA LÍQUIDA (R$)</t>
+        </is>
+      </c>
+      <c r="C10" s="14">
+        <f>C8+C9</f>
+        <v/>
+      </c>
+      <c r="D10" s="14">
+        <f>D8+D9</f>
+        <v/>
+      </c>
+      <c r="E10" s="14">
+        <f>E8+E9</f>
+        <v/>
+      </c>
+      <c r="F10" s="14">
+        <f>F8+F9</f>
+        <v/>
+      </c>
+      <c r="G10" s="14">
+        <f>G8+G9</f>
+        <v/>
+      </c>
+      <c r="H10" s="14">
+        <f>H8+H9</f>
+        <v/>
+      </c>
+      <c r="I10" s="14">
+        <f>I8+I9</f>
+        <v/>
+      </c>
+      <c r="J10" s="14">
+        <f>J8+J9</f>
+        <v/>
+      </c>
+      <c r="K10" s="14">
+        <f>K8+K9</f>
+        <v/>
+      </c>
+      <c r="L10" s="14">
+        <f>L8+L9</f>
+        <v/>
+      </c>
+      <c r="M10" s="14">
+        <f>M8+M9</f>
+        <v/>
+      </c>
+      <c r="N10" s="14">
+        <f>N8+N9</f>
+        <v/>
+      </c>
+      <c r="O10" s="14">
+        <f>O8+O9</f>
+        <v/>
+      </c>
+      <c r="P10" s="14">
+        <f>P8+P9</f>
         <v/>
       </c>
     </row>
@@ -3366,6 +3936,558 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CUSTOS E DESPESAS — 12 ANOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 1</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 2</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 3</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 4</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 5</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 6</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 7</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 8</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 9</t>
+        </is>
+      </c>
+      <c r="L3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 10</t>
+        </is>
+      </c>
+      <c r="M3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 11</t>
+        </is>
+      </c>
+      <c r="N3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 12</t>
+        </is>
+      </c>
+      <c r="O3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 13</t>
+        </is>
+      </c>
+      <c r="P3" s="13" t="inlineStr">
+        <is>
+          <t>Ano 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Custo variável de produção (R$)</t>
+        </is>
+      </c>
+      <c r="C4" s="19">
+        <f>Producao_Receita!C4*Premissas!C$21</f>
+        <v/>
+      </c>
+      <c r="D4" s="19">
+        <f>Producao_Receita!D4*Premissas!D$21</f>
+        <v/>
+      </c>
+      <c r="E4" s="19">
+        <f>Producao_Receita!E4*Premissas!E$21</f>
+        <v/>
+      </c>
+      <c r="F4" s="19">
+        <f>Producao_Receita!F4*Premissas!F$21</f>
+        <v/>
+      </c>
+      <c r="G4" s="19">
+        <f>Producao_Receita!G4*Premissas!G$21</f>
+        <v/>
+      </c>
+      <c r="H4" s="19">
+        <f>Producao_Receita!H4*Premissas!H$21</f>
+        <v/>
+      </c>
+      <c r="I4" s="19">
+        <f>Producao_Receita!I4*Premissas!I$21</f>
+        <v/>
+      </c>
+      <c r="J4" s="19">
+        <f>Producao_Receita!J4*Premissas!J$21</f>
+        <v/>
+      </c>
+      <c r="K4" s="19">
+        <f>Producao_Receita!K4*Premissas!K$21</f>
+        <v/>
+      </c>
+      <c r="L4" s="19">
+        <f>Producao_Receita!L4*Premissas!L$21</f>
+        <v/>
+      </c>
+      <c r="M4" s="19">
+        <f>Producao_Receita!M4*Premissas!M$21</f>
+        <v/>
+      </c>
+      <c r="N4" s="19">
+        <f>Producao_Receita!N4*Premissas!N$21</f>
+        <v/>
+      </c>
+      <c r="O4" s="19">
+        <f>Producao_Receita!O4*Premissas!O$21</f>
+        <v/>
+      </c>
+      <c r="P4" s="19">
+        <f>Producao_Receita!P4*Premissas!P$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Custo do frete próprio (R$)</t>
+        </is>
+      </c>
+      <c r="C5" s="19">
+        <f>Producao_Receita!C7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="D5" s="19">
+        <f>Producao_Receita!D7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="E5" s="19">
+        <f>Producao_Receita!E7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="F5" s="19">
+        <f>Producao_Receita!F7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="G5" s="19">
+        <f>Producao_Receita!G7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="H5" s="19">
+        <f>Producao_Receita!H7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="I5" s="19">
+        <f>Producao_Receita!I7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="J5" s="19">
+        <f>Producao_Receita!J7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="K5" s="19">
+        <f>Producao_Receita!K7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="L5" s="19">
+        <f>Producao_Receita!L7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="M5" s="19">
+        <f>Producao_Receita!M7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="N5" s="19">
+        <f>Producao_Receita!N7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="O5" s="19">
+        <f>Producao_Receita!O7*Premissas!$B$16</f>
+        <v/>
+      </c>
+      <c r="P5" s="19">
+        <f>Producao_Receita!P7*Premissas!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>CFEM (R$)</t>
+        </is>
+      </c>
+      <c r="C6" s="19">
+        <f>Producao_Receita!C8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="D6" s="19">
+        <f>Producao_Receita!D8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="E6" s="19">
+        <f>Producao_Receita!E8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="F6" s="19">
+        <f>Producao_Receita!F8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="G6" s="19">
+        <f>Producao_Receita!G8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="H6" s="19">
+        <f>Producao_Receita!H8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="I6" s="19">
+        <f>Producao_Receita!I8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="J6" s="19">
+        <f>Producao_Receita!J8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="K6" s="19">
+        <f>Producao_Receita!K8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="L6" s="19">
+        <f>Producao_Receita!L8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="M6" s="19">
+        <f>Producao_Receita!M8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="N6" s="19">
+        <f>Producao_Receita!N8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="O6" s="19">
+        <f>Producao_Receita!O8*Premissas!$B$18</f>
+        <v/>
+      </c>
+      <c r="P6" s="19">
+        <f>Producao_Receita!P8*Premissas!$B$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Custos fixos de produção (R$)</t>
+        </is>
+      </c>
+      <c r="C7" s="19">
+        <f>Premissas!C$22</f>
+        <v/>
+      </c>
+      <c r="D7" s="19">
+        <f>Premissas!D$22</f>
+        <v/>
+      </c>
+      <c r="E7" s="19">
+        <f>Premissas!E$22</f>
+        <v/>
+      </c>
+      <c r="F7" s="19">
+        <f>Premissas!F$22</f>
+        <v/>
+      </c>
+      <c r="G7" s="19">
+        <f>Premissas!G$22</f>
+        <v/>
+      </c>
+      <c r="H7" s="19">
+        <f>Premissas!H$22</f>
+        <v/>
+      </c>
+      <c r="I7" s="19">
+        <f>Premissas!I$22</f>
+        <v/>
+      </c>
+      <c r="J7" s="19">
+        <f>Premissas!J$22</f>
+        <v/>
+      </c>
+      <c r="K7" s="19">
+        <f>Premissas!K$22</f>
+        <v/>
+      </c>
+      <c r="L7" s="19">
+        <f>Premissas!L$22</f>
+        <v/>
+      </c>
+      <c r="M7" s="19">
+        <f>Premissas!M$22</f>
+        <v/>
+      </c>
+      <c r="N7" s="19">
+        <f>Premissas!N$22</f>
+        <v/>
+      </c>
+      <c r="O7" s="19">
+        <f>Premissas!O$22</f>
+        <v/>
+      </c>
+      <c r="P7" s="19">
+        <f>Premissas!P$22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Despesas adm/com/trib (R$)</t>
+        </is>
+      </c>
+      <c r="C8" s="19">
+        <f>Premissas!C$23</f>
+        <v/>
+      </c>
+      <c r="D8" s="19">
+        <f>Premissas!D$23</f>
+        <v/>
+      </c>
+      <c r="E8" s="19">
+        <f>Premissas!E$23</f>
+        <v/>
+      </c>
+      <c r="F8" s="19">
+        <f>Premissas!F$23</f>
+        <v/>
+      </c>
+      <c r="G8" s="19">
+        <f>Premissas!G$23</f>
+        <v/>
+      </c>
+      <c r="H8" s="19">
+        <f>Premissas!H$23</f>
+        <v/>
+      </c>
+      <c r="I8" s="19">
+        <f>Premissas!I$23</f>
+        <v/>
+      </c>
+      <c r="J8" s="19">
+        <f>Premissas!J$23</f>
+        <v/>
+      </c>
+      <c r="K8" s="19">
+        <f>Premissas!K$23</f>
+        <v/>
+      </c>
+      <c r="L8" s="19">
+        <f>Premissas!L$23</f>
+        <v/>
+      </c>
+      <c r="M8" s="19">
+        <f>Premissas!M$23</f>
+        <v/>
+      </c>
+      <c r="N8" s="19">
+        <f>Premissas!N$23</f>
+        <v/>
+      </c>
+      <c r="O8" s="19">
+        <f>Premissas!O$23</f>
+        <v/>
+      </c>
+      <c r="P8" s="19">
+        <f>Premissas!P$23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Custeio grupo (R$)</t>
+        </is>
+      </c>
+      <c r="C9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="D9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="E9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="F9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="G9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="H9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="I9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="J9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="K9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="L9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="M9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="N9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="O9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+      <c r="P9" s="19">
+        <f>Premissas!$B$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL CUSTOS E DESPESAS (R$)</t>
+        </is>
+      </c>
+      <c r="C10" s="19">
+        <f>SUM(C4:C9)</f>
+        <v/>
+      </c>
+      <c r="D10" s="19">
+        <f>SUM(D4:D9)</f>
+        <v/>
+      </c>
+      <c r="E10" s="19">
+        <f>SUM(E4:E9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="19">
+        <f>SUM(F4:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="19">
+        <f>SUM(G4:G9)</f>
+        <v/>
+      </c>
+      <c r="H10" s="19">
+        <f>SUM(H4:H9)</f>
+        <v/>
+      </c>
+      <c r="I10" s="19">
+        <f>SUM(I4:I9)</f>
+        <v/>
+      </c>
+      <c r="J10" s="19">
+        <f>SUM(J4:J9)</f>
+        <v/>
+      </c>
+      <c r="K10" s="19">
+        <f>SUM(K4:K9)</f>
+        <v/>
+      </c>
+      <c r="L10" s="19">
+        <f>SUM(L4:L9)</f>
+        <v/>
+      </c>
+      <c r="M10" s="19">
+        <f>SUM(M4:M9)</f>
+        <v/>
+      </c>
+      <c r="N10" s="19">
+        <f>SUM(N4:N9)</f>
+        <v/>
+      </c>
+      <c r="O10" s="19">
+        <f>SUM(O4:O9)</f>
+        <v/>
+      </c>
+      <c r="P10" s="19">
+        <f>SUM(P4:P9)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3791,7 +4913,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4595,7 +5717,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5098,234 +6220,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>CAPACIDADE DE PAGAMENTO — MOTOR OFICIAL BNB (janela 30–50%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Rédito = Receita BRUTA × (1 − custo padrão). Valores calculados no algoritmo VBA real do banco (script da consultoria, validado ao centésimo). Custo padrão proposto: 68,62% (DRE real PVV); tabela indústria: 67,77% — VALIDAR com o analista.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Configuração</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Comprometimento máx.</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Veredito</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Observação</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Pleito R$ 24,29 mi · 14a · 2 car + 12 amort · receita ultra-conservadora</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="n">
-        <v>0.5095582712098438</v>
-      </c>
-      <c r="C5" s="26" t="inlineStr">
-        <is>
-          <t>NÃO PASSA</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>51,0% — 1 p.p. fora; fecha com preço R$ 74/t (46,5%), platô antecipado (49,8%) ou 95% (42,0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Pleito R$ 24,29 mi · 14a · 2 car + 12 amort · preço R$ 82/t</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="n">
-        <v>0.413330734071942</v>
-      </c>
-      <c r="C6" s="27" t="inlineStr">
-        <is>
-          <t>PASSA</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>41,3% — colchão</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Pleito R$ 24,29 mi · 14a · 2 car + 12 amort · produção 95% da licença</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="n">
-        <v>0.4195555249059341</v>
-      </c>
-      <c r="C7" s="27" t="inlineStr">
-        <is>
-          <t>PASSA</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>42,0% — colchão</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Pleito R$ 24,29 mi · 14a · 3 car + 11 amort · receita-base</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="n">
-        <v>0.5449953606863867</v>
-      </c>
-      <c r="C8" s="26" t="inlineStr">
-        <is>
-          <t>NÃO PASSA</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>54,5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Pleito R$ 24,29 mi · 14a · 4 car + 10 amort · receita-base</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="n">
-        <v>0.6010854034324153</v>
-      </c>
-      <c r="C9" s="26" t="inlineStr">
-        <is>
-          <t>NÃO PASSA</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>60,1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Pleito R$ 24,29 mi · 12a/3c · receita-base (sem condição Mulher)</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="n">
-        <v>0.6700428550535171</v>
-      </c>
-      <c r="C10" s="26" t="inlineStr">
-        <is>
-          <t>NÃO PASSA</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>67,0% — referência</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>FINANCIAMENTO MÁXIMO QUE PASSA (≤50%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>14a · 2c+12a · receita-base</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="n">
-        <v>23964142.38999998</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>14a · 2c+12a · preço R$ 82/t</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="n">
-        <v>27958836.32254746</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>14a · 2c+12a · produção 95% da licença</t>
-        </is>
-      </c>
-      <c r="B15" s="14" t="n">
-        <v>27660200.76147405</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>14a · 4c+10a · receita-base (comparação)</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="n">
-        <v>21200497.68732259</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Formulas sem cache: o Excel recalcula ao abrir. Nota: valores estáticos (o algoritmo do banco não é replicável em fórmula de planilha). Para recalcular após mudar premissas, rodar o script capacidade_pagamento.py da skill do consultor.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Remove framing de 'pedreira-modelo/replica' dos documentos bancários
- Carta §1: 'servirá de modelo operacional e comercial' → pedreira em atividade
  com mesmo processo e portfólio (fato, sem convite a benchmark)
- Estudo de Mercado v3 (novo): 3 trechos em vermelho — 'replica o modelo',
  'replica o catálogo' e 'operação-espelho' neutralizados
- Viabilidade_CIPREM.xlsx: aviso USO INTERNO no LEIA-ME (não anexar ao BNB)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DqEaERD1LDFtugtNrL73cp
</commit_message>
<xml_diff>
--- a/Viabilidade_CIPREM.xlsx
+++ b/Viabilidade_CIPREM.xlsx
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -556,117 +556,124 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr"/>
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t>USO INTERNO — ferramenta de trabalho da consultoria (contém dados de benchmark de outra empresa do grupo). NÃO anexar ao processo BNB: os documentos entregues ao banco não citam esta base de comparação.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>COMO USAR: edite SOMENTE as células AZUIS da aba "Premissas" (as amarelas são as premissas-chave a validar).</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Todas as demais abas recalculam automaticamente. Não edite células pretas (fórmulas) nem verdes (links entre abas).</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
-    </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>ABAS: Premissas → entradas | DRE_PVV_2025 → benchmark real | Producao_Receita / Custos / DRE_Projetada → projeção 12 anos</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>FNE_SAC → financiamento | Fluxo_Indicadores → TIR, VPL, payback, DSCR | Capacidade_BNB → janela 30-50% (motor oficial)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>FNE_SAC → financiamento | Fluxo_Indicadores → TIR, VPL, payback, DSCR | Capacidade_BNB → janela 30-50% (motor oficial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>Sensibilidade → resumo dos cenários prontos (inclui 95% da licença) + produção necessária por ano (DSCR 1,0/1,2/1,3).</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>TRÊS AVISOS IMPORTANTES:</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>1) CUSTO PADRÃO BNB: calculado da DRE real da PVV = 68,62% (tabela indústria BNB: 67,77%). VALIDAR com o analista antes do protocolo.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2) CAPACIDADE: prazo de 14 anos (condição FNE Mulher) montado como 2 de carência + 12 de amortização: o pleito integral</t>
+          <t>1) CUSTO PADRÃO BNB: calculado da DRE real da PVV = 68,62% (tabela indústria BNB: 67,77%). VALIDAR com o analista antes do protocolo.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">   na taxa real (10,3493%) a receita ultra-conservadora fica em 51,0% (1 p.p. fora da janela): o pleito fecha com preço R$ 74/t (46,5%),</t>
+          <t>2) CAPACIDADE: prazo de 14 anos (condição FNE Mulher) montado como 2 de carência + 12 de amortização: o pleito integral</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">   R$ 82/t (41,3%), platô antecipado ao ano 3 (49,8%) ou 95% da licença (42,0%). Colchões não contados: bônus de adimplência (48,2%) e custo padrão tabela (49,1%).</t>
+          <t xml:space="preserve">   na taxa real (10,3493%) a receita ultra-conservadora fica em 51,0% (1 p.p. fora da janela): o pleito fecha com preço R$ 74/t (46,5%),</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>3) LASTRO DE RESERVA: a reserva medida no PAE (480.591 m³) esgota no ano 8 do ramp. O platô de 216 mil t/ano exige nova cubagem</t>
+          <t xml:space="preserve">   R$ 82/t (41,3%), platô antecipado ao ano 3 (49,8%) ou 95% da licença (42,0%). Colchões não contados: bônus de adimplência (48,2%) e custo padrão tabela (49,1%).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>3) LASTRO DE RESERVA: a reserva medida no PAE (480.591 m³) esgota no ano 8 do ramp. O platô de 216 mil t/ano exige nova cubagem</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">   (ver relatório de verificação de licenças, §4). O cenário "reserva_atual" da aba Sensibilidade mostra o efeito de não resolver.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>FONTES: DRE 2025 PVV (BI + Wshare), DADOS_PARA_CIPREM.xlsx (produção/vendas/preços/custos/insumos/pessoal),</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>plano de produção e pesquisa de preços ES desta consultoria (SINAPI-ES 06/2026, DER-ES), orçamento de implantação 19/06/2026.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>plano de produção e pesquisa de preços ES desta consultoria (SINAPI-ES 06/2026, DER-ES), orçamento de implantação 19/06/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Mix_Produtos → de onde vem o R$/t: mix real da PVV linha a linha, reconciliação até o caso-base (R$ 68,50) e verificação produto a produto da carta consulta.</t>
         </is>

</xml_diff>